<commit_message>
Polish Excel M01 L02 workbook objectives
</commit_message>
<xml_diff>
--- a/EXCEL/M01/bus123-excel-m01-l02-starter.xlsx
+++ b/EXCEL/M01/bus123-excel-m01-l02-starter.xlsx
@@ -642,7 +642,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>I can create a worksheet with clear labels and consistent structure.</t>
+          <t>I can format worksheet labels, values, and totals so the data is easier to read.</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>I can enter and edit business data accurately.</t>
+          <t>I can organize rows and columns without changing the meaning of the data.</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,14 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>I can use basic spreadsheet formulas to check my work.</t>
+          <t>I can apply consistent number formats for business values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>I can prepare a worksheet for another business user to review.</t>
         </is>
       </c>
     </row>
@@ -745,8 +752,6 @@
           <t>Tidal Goods Co.</t>
         </is>
       </c>
-      <c r="E1" s="6" t="n"/>
-      <c r="H1" s="6" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -754,8 +759,6 @@
           <t>Main Activity: Format and Organize a Product Worksheet</t>
         </is>
       </c>
-      <c r="E2" s="6" t="n"/>
-      <c r="H2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="E3" s="6" t="n"/>
@@ -952,17 +955,9 @@
           <t>Use filters or sorting to identify which items are in the High reorder group. Keep product labels visible and number formats consistent.</t>
         </is>
       </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="H13" s="6" t="n"/>
-    </row>
-    <row r="14">
-      <c r="E14" s="6" t="n"/>
-      <c r="H14" s="6" t="n"/>
-    </row>
-    <row r="15">
-      <c r="E15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
-    </row>
+    </row>
+    <row r="14"/>
+    <row r="15"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:J1"/>

</xml_diff>